<commit_message>
Corregir layout del informe (leyendas inline) y preservar PDF/capturas al renderizar.
Evita que la codificación por color parta párrafos (p.ej. 2.3.2), endurece fill/render del informe y deja documentado el ciclo UI/pipeline/IEEE.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/input/feeders/PA217/Control_Simulacion.xlsx
+++ b/data/input/feeders/PA217/Control_Simulacion.xlsx
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6038</v>
+        <v>9537.879999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2588</v>
+        <v>2587.65</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -705,7 +705,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-20 UI</t>
+          <t>3/03/2026 10:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Anclar §1–§5 a la sesión CYMDIST viva y ejecutar LoadFlow por COM.
Evita Access Violation de CymPy en flujos 5.1/5.2, sincroniza BD+estudio del contexto UI y deja distribución/SpotLoad alineados al motor COM de §3.3.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/input/feeders/PA217/Control_Simulacion.xlsx
+++ b/data/input/feeders/PA217/Control_Simulacion.xlsx
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9537.879999999999</v>
+        <v>2565.9541</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2587.65</v>
+        <v>696.1496</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>

</xml_diff>